<commit_message>
Feature: Add file upload, duplicate room validation, and timestamps in feedback.
</commit_message>
<xml_diff>
--- a/pages/room_schedule.xlsx
+++ b/pages/room_schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yungk\Desktop\NSCC\Projects\Vacant Notification Project\VacNoti\pages\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57A11DB8-DD6A-481C-B4C7-89FAED41ADF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA7D1B8B-8CBD-4E49-B5F0-D57FA6206724}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10403" yWindow="2850" windowWidth="21600" windowHeight="11332" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9760" yWindow="21490" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="roomNum" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>7/F</t>
   </si>
@@ -80,6 +80,15 @@
   </si>
   <si>
     <t>YKK</t>
+  </si>
+  <si>
+    <t>RA1</t>
+  </si>
+  <si>
+    <t>RA2</t>
+  </si>
+  <si>
+    <t>RA3</t>
   </si>
 </sst>
 </file>
@@ -1306,14 +1315,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F5407CB-C67E-4C69-B3B3-746A73826D8B}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:W6"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="19.3984375" customWidth="1"/>
     <col min="3" max="3" width="18.46484375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -1324,7 +1333,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -1341,13 +1350,43 @@
         <v>1703</v>
       </c>
       <c r="F2">
-        <v>1801</v>
+        <v>1704</v>
       </c>
       <c r="G2">
-        <v>1808</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+        <v>1705</v>
+      </c>
+      <c r="H2">
+        <v>1706</v>
+      </c>
+      <c r="I2">
+        <v>1707</v>
+      </c>
+      <c r="J2">
+        <v>1708</v>
+      </c>
+      <c r="K2">
+        <v>1709</v>
+      </c>
+      <c r="L2">
+        <v>1710</v>
+      </c>
+      <c r="M2">
+        <v>1711</v>
+      </c>
+      <c r="N2">
+        <v>1712</v>
+      </c>
+      <c r="O2">
+        <v>1713</v>
+      </c>
+      <c r="P2">
+        <v>1714</v>
+      </c>
+      <c r="W2">
+        <v>1421</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -1355,13 +1394,235 @@
         <v>23455324</v>
       </c>
       <c r="C3">
-        <v>1704</v>
+        <v>1801</v>
       </c>
       <c r="D3">
-        <v>1708</v>
+        <v>1802</v>
       </c>
       <c r="E3">
+        <v>1803</v>
+      </c>
+      <c r="F3">
+        <v>1804</v>
+      </c>
+      <c r="G3">
+        <v>1805</v>
+      </c>
+      <c r="H3">
+        <v>1806</v>
+      </c>
+      <c r="I3">
+        <v>1807</v>
+      </c>
+      <c r="J3">
+        <v>1808</v>
+      </c>
+      <c r="K3">
+        <v>1809</v>
+      </c>
+      <c r="L3">
+        <v>1810</v>
+      </c>
+      <c r="M3">
+        <v>1811</v>
+      </c>
+      <c r="N3">
+        <v>1812</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4">
+        <v>123</v>
+      </c>
+      <c r="C4">
         <v>1901</v>
+      </c>
+      <c r="D4">
+        <v>1902</v>
+      </c>
+      <c r="E4">
+        <v>1903</v>
+      </c>
+      <c r="F4">
+        <v>1904</v>
+      </c>
+      <c r="G4">
+        <v>1905</v>
+      </c>
+      <c r="H4">
+        <v>1906</v>
+      </c>
+      <c r="I4">
+        <v>1907</v>
+      </c>
+      <c r="J4">
+        <v>1908</v>
+      </c>
+      <c r="K4">
+        <v>1909</v>
+      </c>
+      <c r="L4">
+        <v>1910</v>
+      </c>
+      <c r="M4">
+        <v>1911</v>
+      </c>
+      <c r="N4">
+        <v>1912</v>
+      </c>
+      <c r="O4">
+        <v>1913</v>
+      </c>
+      <c r="P4">
+        <v>1914</v>
+      </c>
+      <c r="Q4">
+        <v>1915</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5">
+        <v>456</v>
+      </c>
+      <c r="C5">
+        <v>1501</v>
+      </c>
+      <c r="D5">
+        <v>1502</v>
+      </c>
+      <c r="E5">
+        <v>1503</v>
+      </c>
+      <c r="F5">
+        <v>1504</v>
+      </c>
+      <c r="G5">
+        <v>1505</v>
+      </c>
+      <c r="H5">
+        <v>1506</v>
+      </c>
+      <c r="I5">
+        <v>1507</v>
+      </c>
+      <c r="J5">
+        <v>1508</v>
+      </c>
+      <c r="K5">
+        <v>1509</v>
+      </c>
+      <c r="L5">
+        <v>1510</v>
+      </c>
+      <c r="M5">
+        <v>1511</v>
+      </c>
+      <c r="N5">
+        <v>1512</v>
+      </c>
+      <c r="O5">
+        <v>1513</v>
+      </c>
+      <c r="P5">
+        <v>1514</v>
+      </c>
+      <c r="Q5">
+        <v>1515</v>
+      </c>
+      <c r="R5">
+        <v>1516</v>
+      </c>
+      <c r="S5">
+        <v>1517</v>
+      </c>
+      <c r="T5">
+        <v>1518</v>
+      </c>
+      <c r="U5">
+        <v>1519</v>
+      </c>
+      <c r="V5">
+        <v>1520</v>
+      </c>
+      <c r="W5">
+        <v>1521</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6">
+        <v>789</v>
+      </c>
+      <c r="C6">
+        <v>1401</v>
+      </c>
+      <c r="D6">
+        <v>1402</v>
+      </c>
+      <c r="E6">
+        <v>1403</v>
+      </c>
+      <c r="F6">
+        <v>1404</v>
+      </c>
+      <c r="G6">
+        <v>1405</v>
+      </c>
+      <c r="H6">
+        <v>1406</v>
+      </c>
+      <c r="I6">
+        <v>1407</v>
+      </c>
+      <c r="J6">
+        <v>1408</v>
+      </c>
+      <c r="K6">
+        <v>1409</v>
+      </c>
+      <c r="L6">
+        <v>1410</v>
+      </c>
+      <c r="M6">
+        <v>1411</v>
+      </c>
+      <c r="N6">
+        <v>1412</v>
+      </c>
+      <c r="O6">
+        <v>1413</v>
+      </c>
+      <c r="P6">
+        <v>1414</v>
+      </c>
+      <c r="Q6">
+        <v>1415</v>
+      </c>
+      <c r="R6">
+        <v>1416</v>
+      </c>
+      <c r="S6">
+        <v>1417</v>
+      </c>
+      <c r="T6">
+        <v>1418</v>
+      </c>
+      <c r="U6">
+        <v>1419</v>
+      </c>
+      <c r="V6">
+        <v>1420</v>
+      </c>
+      <c r="W6">
+        <v>1421</v>
       </c>
     </row>
   </sheetData>

</xml_diff>